<commit_message>
meaning_of_colors.xlsx to enlarge copy #
</commit_message>
<xml_diff>
--- a/meaning_of_colors.xlsx
+++ b/meaning_of_colors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gordo893\Documents\bioinformatics\2025\fastcn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB2AA7CF-7565-43B2-B562-86CD1C2B7CA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51B3995B-BB1D-4393-B37E-AB91D386A414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="460" yWindow="0" windowWidth="17900" windowHeight="9785" xr2:uid="{FBA50375-6D60-41E6-A33E-AE0E101D2E7E}"/>
+    <workbookView xWindow="700" yWindow="295" windowWidth="17900" windowHeight="9785" xr2:uid="{FBA50375-6D60-41E6-A33E-AE0E101D2E7E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -102,9 +102,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="26"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -131,9 +139,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2868,249 +2879,251 @@
   <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="50" customHeight="1" x14ac:dyDescent="0.75"/>
   <cols>
+    <col min="1" max="1" width="8.7265625" style="2"/>
     <col min="2" max="3" width="13.40625" customWidth="1"/>
+    <col min="4" max="4" width="8.7265625" style="2"/>
     <col min="5" max="5" width="7.2265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A1">
+      <c r="A1" s="2">
         <v>0</v>
       </c>
       <c r="B1" s="1">
         <v>229229229</v>
       </c>
-      <c r="D1">
+      <c r="D1" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A2">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A3">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>1</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="2">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A4">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A5">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="2">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A6">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A7">
+      <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="2">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A8">
+      <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="2">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A9">
+      <c r="A9" s="2">
         <v>8</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="2">
         <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A10">
+      <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>8</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="2">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A11">
+      <c r="A11" s="2">
         <v>10</v>
       </c>
       <c r="B11" t="s">
         <v>9</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A12">
+      <c r="A12" s="2">
         <v>20</v>
       </c>
       <c r="B12" t="s">
         <v>10</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="2">
         <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A13">
+      <c r="A13" s="2">
         <v>30</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="2">
         <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A14">
+      <c r="A14" s="2">
         <v>40</v>
       </c>
       <c r="B14" t="s">
         <v>12</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="2">
         <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A15">
+      <c r="A15" s="2">
         <v>50</v>
       </c>
       <c r="B15" t="s">
         <v>13</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="2">
         <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A16">
+      <c r="A16" s="2">
         <v>60</v>
       </c>
       <c r="B16" t="s">
         <v>14</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="2">
         <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A17">
+      <c r="A17" s="2">
         <v>70</v>
       </c>
       <c r="B17" t="s">
         <v>15</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="2">
         <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A18">
+      <c r="A18" s="2">
         <v>80</v>
       </c>
       <c r="B18" t="s">
         <v>16</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="2">
         <v>80</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A19">
+      <c r="A19" s="2">
         <v>90</v>
       </c>
       <c r="B19" t="s">
         <v>17</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="2">
         <v>90</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A20">
+      <c r="A20" s="2">
         <v>100</v>
       </c>
       <c r="B20" t="s">
         <v>18</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="2">
         <v>100</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A21">
+      <c r="A21" s="2">
         <v>110</v>
       </c>
       <c r="B21" t="s">
         <v>19</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="2">
         <v>110</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A22">
+      <c r="A22" s="2">
         <v>120</v>
       </c>
       <c r="B22" s="1">
         <v>255192203</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="2">
         <v>120</v>
       </c>
     </row>

</xml_diff>